<commit_message>
Methods from the clause naming the variable; pH chemical names; warn when pypdf is missing; regenerate outputs
Outputs of all 74 written variables with the last-resort id order, and soil pH with the method fixes (10.15485/1577267 pH_H2O, 10.5440/1618325 pH_KCl).
</commit_message>
<xml_diff>
--- a/data/processed/harmonization/Acidity__Soil_pH/10.15485_1618870/10.15485_1618870_soil_Acidity__Soil_pH.xlsx
+++ b/data/processed/harmonization/Acidity__Soil_pH/10.15485_1618870/10.15485_1618870_soil_Acidity__Soil_pH.xlsx
@@ -426,13 +426,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -440,7 +440,8 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,6 +502,11 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>source_row</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
@@ -518,12 +524,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>El Verde:Ridge:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -547,9 +553,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -566,12 +575,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>El Verde:Ridge:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -595,9 +604,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -614,12 +626,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>El Verde:Ridge:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -643,9 +655,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -662,12 +677,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>El Verde:Ridge:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -691,9 +706,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -710,12 +728,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>El Verde:Ridge:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -739,9 +757,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -758,12 +779,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>El Verde:Ridge:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -787,9 +808,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L7" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -806,12 +830,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>El Verde:Slope:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -835,9 +859,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -854,12 +881,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>El Verde:Slope:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -883,9 +910,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L9" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -902,12 +932,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>El Verde:Slope:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -931,9 +961,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L10" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -950,12 +983,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>El Verde:Slope:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -979,9 +1012,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L11" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -998,12 +1034,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>El Verde:Slope:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1027,9 +1063,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L12" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1085,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>El Verde:Slope:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -1075,9 +1114,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L13" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1136,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>El Verde:Slope:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -1123,9 +1165,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L14" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1142,12 +1187,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>El Verde:Slope:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -1171,9 +1216,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L15" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1190,12 +1238,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>El Verde:Slope:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -1219,9 +1267,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L16" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1289,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>El Verde:Slope:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -1267,9 +1318,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1286,12 +1340,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>El Verde:Slope:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -1315,9 +1369,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L18" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1391,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>El Verde:Slope:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
@@ -1363,9 +1420,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L19" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1382,12 +1442,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>El Verde:Valley:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -1411,9 +1471,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1493,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>El Verde:Valley:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -1459,9 +1522,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L21" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1544,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>El Verde:Valley:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
@@ -1507,9 +1573,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L22" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1595,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>El Verde:Valley:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
@@ -1555,9 +1624,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L23" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1646,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>El Verde:Valley:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
@@ -1603,9 +1675,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L24" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1622,12 +1697,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>El Verde:Ridge:a:1:2017-08-01</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
@@ -1651,9 +1726,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L25" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1670,12 +1748,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>El Verde:Ridge:b:1:2017-08-01</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
@@ -1699,9 +1777,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L26" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1718,12 +1799,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>El Verde:Ridge:a:2:2017-08-01</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
@@ -1747,9 +1828,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L27" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1850,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>El Verde:Ridge:b:2:2017-08-01</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -1795,9 +1879,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L28" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1901,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>El Verde:Ridge:a:3:2017-08-01</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -1843,9 +1930,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L29" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1862,12 +1952,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>El Verde:Ridge:b:3:2017-08-01</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
@@ -1891,9 +1981,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L30" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1910,12 +2003,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>El Verde:Valley:a:1:2017-08-01</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -1939,9 +2032,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L31" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -1958,12 +2054,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>El Verde:Valley:b:1:2017-08-01</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -1987,9 +2083,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L32" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2006,12 +2105,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>El Verde:Valley:a:2:2017-08-01</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -2035,9 +2134,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L33" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2156,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>El Verde:Valley:b:2:2017-08-01</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
@@ -2083,9 +2185,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L34" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2102,12 +2207,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>El Verde:Valley:a:3:2017-08-01</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2131,9 +2236,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L35" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2150,12 +2258,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>El Verde:Valley:b:3:2017-08-01</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -2179,9 +2287,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L36" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2198,12 +2309,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>El Verde:Ridge:a:1:NA</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2223,9 +2334,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L37" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2242,12 +2356,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>El Verde:Ridge:b:1:NA</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
@@ -2267,9 +2381,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L38" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2403,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>El Verde:Ridge:a:2:NA</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2311,9 +2428,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L39" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2330,12 +2450,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>El Verde:Ridge:b:2:NA</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr"/>
@@ -2355,9 +2475,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L40" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2374,12 +2497,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>El Verde:Ridge:a:3:NA</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
@@ -2399,9 +2522,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L41" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2544,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>El Verde:Ridge:b:3:NA</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
@@ -2443,9 +2569,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L42" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2462,12 +2591,12 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>El Verde:Slope:a:1:NA</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2487,9 +2616,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L43" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2506,12 +2638,12 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>El Verde:Slope:b:1:NA</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
@@ -2531,9 +2663,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L44" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2550,12 +2685,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>El Verde:Slope:a:2:NA</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2575,9 +2710,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L45" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2732,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>El Verde:Slope:b:2:NA</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
@@ -2619,9 +2757,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L46" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2779,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>El Verde:Slope:a:3:NA</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2663,9 +2804,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L47" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2826,12 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>El Verde:Slope:b:3:NA</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
@@ -2707,9 +2851,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K48" s="2" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L48" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2726,12 +2873,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>El Verde:Slope:a:1:NA</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2751,9 +2898,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L49" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2770,12 +2920,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>El Verde:Slope:b:1:NA</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
@@ -2795,9 +2945,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L50" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2814,12 +2967,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>El Verde:Slope:a:2:NA</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
@@ -2839,9 +2992,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K51" s="2" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L51" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2858,12 +3014,12 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>El Verde:Slope:b:2:NA</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr"/>
@@ -2883,9 +3039,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L52" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2902,12 +3061,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>El Verde:Slope:a:3:NA</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr"/>
@@ -2927,9 +3086,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L53" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2946,12 +3108,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>El Verde:Slope:b:3:NA</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -2971,9 +3133,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L54" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -2990,12 +3155,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>El Verde:Valley:a:1:NA</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
@@ -3015,9 +3180,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K55" s="2" t="inlineStr"/>
-      <c r="L55" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L55" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3034,12 +3202,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>El Verde:Valley:b:1:NA</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
@@ -3059,9 +3227,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L56" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3078,12 +3249,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>El Verde:Valley:a:2:NA</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr"/>
@@ -3103,9 +3274,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L57" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3122,12 +3296,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>El Verde:Valley:b:2:NA</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr"/>
@@ -3147,9 +3321,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L58" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3166,12 +3343,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>El Verde:Valley:a:3:NA</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr"/>
@@ -3191,9 +3368,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L59" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3210,12 +3390,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>El Verde:Valley:b:3:NA</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr"/>
@@ -3235,9 +3415,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L60" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3254,12 +3437,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>El Verde:Ridge:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr"/>
@@ -3283,9 +3466,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L61" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3302,12 +3488,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>El Verde:Ridge:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr"/>
@@ -3331,9 +3517,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L62" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3350,12 +3539,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>El Verde:Slope:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr"/>
@@ -3379,9 +3568,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L63" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3398,12 +3590,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>El Verde:Slope:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
@@ -3427,9 +3619,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L64" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3446,12 +3641,12 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>El Verde:Slope:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr"/>
@@ -3475,9 +3670,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K65" s="2" t="inlineStr"/>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L65" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3692,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>El Verde:Slope:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr"/>
@@ -3523,9 +3721,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L66" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3542,12 +3743,12 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>El Verde:Valley:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr"/>
@@ -3571,9 +3772,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L67" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3590,12 +3794,12 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>El Verde:Valley:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr"/>
@@ -3619,9 +3823,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L68" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3638,12 +3845,12 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>El Verde:Ridge:a:1:2018-05-01</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr"/>
@@ -3667,9 +3874,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L69" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3686,12 +3896,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>El Verde:Ridge:b:1:2018-05-01</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr"/>
@@ -3715,9 +3925,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L70" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3734,12 +3947,12 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>El Verde:Valley:a:1:2018-05-01</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr"/>
@@ -3763,9 +3976,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L71" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3782,12 +3998,12 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>El Verde:Valley:b:1:2018-05-01</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr"/>
@@ -3811,9 +4027,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O</t>
+      <c r="L72" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_H2O; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3830,12 +4049,12 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>El Verde:Ridge:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr"/>
@@ -3859,9 +4078,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3878,12 +4100,12 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>El Verde:Ridge:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr"/>
@@ -3907,9 +4129,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L74" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3926,12 +4151,12 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>El Verde:Ridge:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr"/>
@@ -3955,9 +4180,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K75" s="2" t="inlineStr"/>
-      <c r="L75" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L75" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -3974,12 +4202,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>El Verde:Ridge:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
@@ -4003,9 +4231,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L76" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4022,12 +4253,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>El Verde:Ridge:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
@@ -4051,9 +4282,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L77" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4070,12 +4304,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>El Verde:Ridge:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
@@ -4099,9 +4333,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L78" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4118,12 +4355,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>El Verde:Slope:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr"/>
@@ -4147,9 +4384,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
-      <c r="L79" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L79" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4166,12 +4406,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>El Verde:Slope:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr"/>
@@ -4195,9 +4435,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
-      <c r="L80" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L80" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4214,12 +4457,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>El Verde:Slope:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr"/>
@@ -4243,9 +4486,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K81" s="2" t="inlineStr"/>
-      <c r="L81" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L81" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4508,12 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>El Verde:Slope:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr"/>
@@ -4291,9 +4537,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K82" s="2" t="inlineStr"/>
-      <c r="L82" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L82" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4310,12 +4559,12 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>El Verde:Slope:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
@@ -4339,9 +4588,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K83" s="2" t="inlineStr"/>
-      <c r="L83" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L83" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4358,12 +4610,12 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>El Verde:Slope:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr"/>
@@ -4387,9 +4639,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K84" s="2" t="inlineStr"/>
-      <c r="L84" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L84" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4406,12 +4661,12 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>El Verde:Slope:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr"/>
@@ -4435,9 +4690,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K85" s="2" t="inlineStr"/>
-      <c r="L85" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L85" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4454,12 +4712,12 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>El Verde:Slope:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr"/>
@@ -4483,9 +4741,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K86" s="2" t="inlineStr"/>
-      <c r="L86" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L86" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4502,12 +4763,12 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>El Verde:Slope:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr"/>
@@ -4531,9 +4792,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
-      <c r="L87" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L87" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4550,12 +4814,12 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>El Verde:Slope:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr"/>
@@ -4579,9 +4843,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L88" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4598,12 +4865,12 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>El Verde:Slope:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr"/>
@@ -4627,9 +4894,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L89" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4646,12 +4916,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>El Verde:Slope:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr"/>
@@ -4675,9 +4945,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K90" s="2" t="inlineStr"/>
-      <c r="L90" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L90" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4694,12 +4967,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>El Verde:Valley:a:1:2017-04-01</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr"/>
@@ -4723,9 +4996,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K91" s="2" t="inlineStr"/>
-      <c r="L91" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L91" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4742,12 +5018,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>El Verde:Valley:b:1:2017-04-01</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr"/>
@@ -4771,9 +5047,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L92" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4790,12 +5069,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>El Verde:Valley:a:2:2017-04-01</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr"/>
@@ -4819,9 +5098,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K93" s="2" t="inlineStr"/>
-      <c r="L93" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L93" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4838,12 +5120,12 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>El Verde:Valley:b:2:2017-04-01</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr"/>
@@ -4867,9 +5149,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K94" s="2" t="inlineStr"/>
-      <c r="L94" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L94" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4886,12 +5171,12 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>El Verde:Valley:a:3:2017-04-01</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr"/>
@@ -4915,9 +5200,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K95" s="2" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L95" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4934,12 +5222,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>El Verde:Valley:b:3:2017-04-01</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr"/>
@@ -4963,9 +5251,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K96" s="2" t="inlineStr"/>
-      <c r="L96" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L96" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -4982,12 +5273,12 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>El Verde:Ridge:a:1:2017-08-01</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr"/>
@@ -5011,9 +5302,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
-      <c r="L97" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L97" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5030,12 +5324,12 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>El Verde:Ridge:b:1:2017-08-01</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr"/>
@@ -5059,9 +5353,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K98" s="2" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L98" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5078,12 +5375,12 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>El Verde:Ridge:a:2:2017-08-01</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr"/>
@@ -5107,9 +5404,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K99" s="2" t="inlineStr"/>
-      <c r="L99" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L99" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5126,12 +5426,12 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>El Verde:Ridge:b:2:2017-08-01</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr"/>
@@ -5155,9 +5455,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
-      <c r="L100" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L100" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5174,12 +5477,12 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>El Verde:Ridge:a:3:2017-08-01</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr"/>
@@ -5203,9 +5506,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K101" s="2" t="inlineStr"/>
-      <c r="L101" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L101" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5222,12 +5528,12 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>El Verde:Ridge:b:3:2017-08-01</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr"/>
@@ -5251,9 +5557,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K102" s="2" t="inlineStr"/>
-      <c r="L102" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L102" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5270,12 +5579,12 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>El Verde:Valley:a:1:2017-08-01</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr"/>
@@ -5299,9 +5608,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K103" s="2" t="inlineStr"/>
-      <c r="L103" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L103" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5318,12 +5630,12 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>El Verde:Valley:b:1:2017-08-01</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr"/>
@@ -5347,9 +5659,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K104" s="2" t="inlineStr"/>
-      <c r="L104" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L104" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5366,12 +5681,12 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>El Verde:Valley:a:2:2017-08-01</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr"/>
@@ -5395,9 +5710,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K105" s="2" t="inlineStr"/>
-      <c r="L105" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L105" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5414,12 +5732,12 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>El Verde:Valley:b:2:2017-08-01</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr"/>
@@ -5443,9 +5761,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K106" s="2" t="inlineStr"/>
-      <c r="L106" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L106" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5462,12 +5783,12 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>El Verde:Valley:a:3:2017-08-01</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr"/>
@@ -5491,9 +5812,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K107" s="2" t="inlineStr"/>
-      <c r="L107" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L107" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5510,12 +5834,12 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>El Verde:Valley:b:3:2017-08-01</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr"/>
@@ -5539,9 +5863,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K108" s="2" t="inlineStr"/>
-      <c r="L108" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L108" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5558,12 +5885,12 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>El Verde:Ridge:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr"/>
@@ -5587,9 +5914,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K109" s="2" t="inlineStr"/>
-      <c r="L109" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L109" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5606,12 +5936,12 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>El Verde:Ridge:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr"/>
@@ -5635,9 +5965,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
-      <c r="L110" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L110" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5654,12 +5987,12 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>El Verde:Slope:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr"/>
@@ -5683,9 +6016,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K111" s="2" t="inlineStr"/>
-      <c r="L111" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L111" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5702,12 +6038,12 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>El Verde:Slope:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr"/>
@@ -5731,9 +6067,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K112" s="2" t="inlineStr"/>
-      <c r="L112" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L112" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5750,12 +6089,12 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>El Verde:Slope:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr"/>
@@ -5779,9 +6118,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K113" s="2" t="inlineStr"/>
-      <c r="L113" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L113" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5798,12 +6140,12 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>El Verde:Slope:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr"/>
@@ -5827,9 +6169,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K114" s="2" t="inlineStr"/>
-      <c r="L114" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L114" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5846,12 +6191,12 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>El Verde:Valley:a:1:2018-01-01</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr"/>
@@ -5875,9 +6220,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K115" s="2" t="inlineStr"/>
-      <c r="L115" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L115" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5894,12 +6242,12 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>El Verde:Valley:b:1:2018-01-01</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr"/>
@@ -5923,9 +6271,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K116" s="2" t="inlineStr"/>
-      <c r="L116" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L116" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5942,12 +6293,12 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>El Verde:Ridge:a:1:2018-05-01</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr"/>
@@ -5971,9 +6322,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
-      <c r="L117" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L117" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -5990,12 +6344,12 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>El Verde:Ridge:b:1:2018-05-01</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr"/>
@@ -6019,9 +6373,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
-      <c r="L118" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L118" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -6038,12 +6395,12 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>El Verde:Valley:a:1:2018-05-01</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr"/>
@@ -6067,9 +6424,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
-      <c r="L119" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L119" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>
@@ -6086,12 +6446,12 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>El Verde:Valley:b:1:2018-05-01</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>source_row</t>
+          <t>Soil Site:Topographic_locations:Lab_replicate:Field_replicate:date</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr"/>
@@ -6115,9 +6475,12 @@
         <v>-65.81948</v>
       </c>
       <c r="K120" s="2" t="inlineStr"/>
-      <c r="L120" s="2" t="inlineStr">
-        <is>
-          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2</t>
+      <c r="L120" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>lat/long source: doi:10.15485/1618870 package spatialCoverage point; source column pH_CaCl2; id not unique: 28 rows share an id</t>
         </is>
       </c>
     </row>

</xml_diff>